<commit_message>
Save library recording Testing HM - e0d149a6-6fd3-4f26-92a6-f468107f57f1 - 2026-10-13T12:09:26.911996Z
</commit_message>
<xml_diff>
--- a/library/projects/qa-sample-app/recordings/e0d149a6-6fd3-4f26-92a6-f468107f57f1/resources/azure-devops.xlsx
+++ b/library/projects/qa-sample-app/recordings/e0d149a6-6fd3-4f26-92a6-f468107f57f1/resources/azure-devops.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,6 +447,34 @@
           <t>Screenshot</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Testing HM</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Open https://www.hm.com/</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>https://www.hm.com/</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>